<commit_message>
Updated the insertMany method
</commit_message>
<xml_diff>
--- a/universities.xlsx
+++ b/universities.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mr\Documents\GitHub\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mr\Desktop\springboot\excel-db-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8589376-D709-44E7-84CA-4346D440ECD4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9603BE95-FAC5-4A38-AE0D-B3EE1D828B82}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{F7E80C4E-4D08-421F-95DD-650FF3B43521}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
   <si>
     <t>id</t>
   </si>
@@ -103,6 +103,27 @@
   </si>
   <si>
     <t>Finance</t>
+  </si>
+  <si>
+    <t>GIKI</t>
+  </si>
+  <si>
+    <t>Electrical Engineering</t>
+  </si>
+  <si>
+    <t>Topi</t>
+  </si>
+  <si>
+    <t>Bahria University</t>
+  </si>
+  <si>
+    <t>Computer Engineering</t>
+  </si>
+  <si>
+    <t>PIEAS</t>
+  </si>
+  <si>
+    <t>Nuclear Engineering</t>
   </si>
 </sst>
 </file>
@@ -454,7 +475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F46A2D5-0A58-487D-9178-ECEE463F0A08}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19.26953125" customWidth="1"/>
@@ -671,6 +692,84 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="G9">
+        <v>300000</v>
+      </c>
+      <c r="H9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10">
+        <v>9</v>
+      </c>
+      <c r="G10">
+        <v>160000</v>
+      </c>
+      <c r="H10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11">
+        <v>10</v>
+      </c>
+      <c r="G11">
+        <v>250000</v>
+      </c>
+      <c r="H11">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>